<commit_message>
docs: atualiza simulacoes de custo FinOps com Job mensal e Job de limpeza
Adiciona os dois workloads que faltavam nas planilhas de custo: Job mensal de
fechamento (ADR-006) e Job de limpeza da Landing Zone com retencao de 30 dias
(ADR-009). Custo residual (~US$0,23/mes somados), sem impacto relevante no
total, mas necessario para a planilha refletir o que os ADRs ja documentam.
Nota adicionada na aba de cenarios explicando por que esses dois jobs nao sao
duplicados por cenario de compute.
</commit_message>
<xml_diff>
--- a/docs/custos/azure_infraestrutura_custo_simulacao.xlsx
+++ b/docs/custos/azure_infraestrutura_custo_simulacao.xlsx
@@ -75,12 +75,24 @@
         </r>
       </text>
     </comment>
+    <comment ref="F7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Referência de mercado — confirmar na calculadora oficial da Azure antes de decisão real.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="64">
   <si>
     <t xml:space="preserve">Simulação — Azure Pricing Calculator (infraestrutura)</t>
   </si>
@@ -170,6 +182,12 @@
   </si>
   <si>
     <t xml:space="preserve">Só se aplica ao cenário Econômico (compute clássico). Em Serverless o custo de VM já está embutido na tarifa DBU — não há bill separado de VM Azure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VM — Job mensal + Job de limpeza (ADR-006, ADR-009)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fechamento mensal (execução única) e limpeza diária da Landing Zone (retenção 30 dias). Custo residual, mesma ressalva de Serverless da linha acima.</t>
   </si>
   <si>
     <t xml:space="preserve">Armazenamento ADLS Gen2 (Hot, LRS)</t>
@@ -894,7 +912,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:H12"/>
+  <dimension ref="A2:H13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -965,77 +983,77 @@
         <v>30</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>24</v>
+        <v>1.55</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F4" s="10" t="n">
-        <v>0.021</v>
+        <v>0.564</v>
       </c>
       <c r="G4" s="11" t="n">
         <f aca="false">D4*F4</f>
-        <v>0.504</v>
+        <v>0.8742</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>0.065</v>
+        <v>0.021</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">D5*F5</f>
-        <v>0.78</v>
+        <v>0.504</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.0052</v>
+        <v>0.065</v>
       </c>
       <c r="G6" s="11" t="n">
         <f aca="false">D6*F6</f>
-        <v>0.26</v>
+        <v>0.78</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>38</v>
@@ -1046,34 +1064,34 @@
         <v>39</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="13" t="n">
-        <v>0</v>
+      <c r="D7" s="9" t="n">
+        <v>50</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0</v>
+        <v>0.0052</v>
       </c>
       <c r="G7" s="11" t="n">
         <f aca="false">D7*F7</f>
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>27</v>
@@ -1082,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>0</v>
@@ -1092,24 +1110,24 @@
         <v>0</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>47</v>
-      </c>
       <c r="C9" s="8" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D9" s="13" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>0</v>
@@ -1119,25 +1137,52 @@
         <v>0</v>
       </c>
       <c r="H9" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="C10" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="15" t="n">
-        <f aca="false">SUM(G3:G9)</f>
-        <v>25.232</v>
+      <c r="F10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <f aca="false">D10*F10</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G12" s="15" t="n">
-        <f aca="false">G11*12</f>
-        <v>302.784</v>
+        <f aca="false">SUM(G3:G10)</f>
+        <v>26.1062</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <f aca="false">G12*12</f>
+        <v>313.2744</v>
       </c>
     </row>
   </sheetData>
@@ -1166,24 +1211,24 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23.69</v>
+        <v>24.56</v>
       </c>
       <c r="C3" s="11" t="n">
         <v>0</v>
@@ -1194,7 +1239,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B4" s="11" t="n">
         <v>0.5</v>
@@ -1208,7 +1253,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>1.04</v>
@@ -1222,7 +1267,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>0</v>
@@ -1236,11 +1281,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">SUM(B3:B6)</f>
-        <v>25.23</v>
+        <v>26.1</v>
       </c>
       <c r="C7" s="16" t="n">
         <f aca="false">SUM(C3:C6)</f>
@@ -1253,11 +1298,11 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" s="16" t="n">
         <f aca="false">B7*12</f>
-        <v>302.76</v>
+        <v>313.2</v>
       </c>
       <c r="C8" s="16" t="n">
         <f aca="false">C7*12</f>
@@ -1270,12 +1315,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>

</xml_diff>